<commit_message>
Mejoras en los modelos
</commit_message>
<xml_diff>
--- a/Docs/ConfiguracionRealModelo.xlsx
+++ b/Docs/ConfiguracionRealModelo.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fabia\Desktop\Universidad\TesisML\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F9227D9-B230-4F29-9DD0-3FEB79183B5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D09349C2-2B85-498C-AD5A-6B547749B796}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{EB321E2F-A158-4D4F-98D8-E5A615C233E9}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{EB321E2F-A158-4D4F-98D8-E5A615C233E9}"/>
   </bookViews>
   <sheets>
     <sheet name="LSTM Clasica " sheetId="1" r:id="rId1"/>
     <sheet name="LSTM Bidireccional" sheetId="2" r:id="rId2"/>
-    <sheet name="Hoja3" sheetId="3" r:id="rId3"/>
+    <sheet name="CNN" sheetId="4" r:id="rId3"/>
+    <sheet name="Hoja3" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="22">
   <si>
     <t>Descripcion</t>
   </si>
@@ -442,10 +443,19 @@
     <t>LSTM Clasica con ventanas de tiempo de 90 dias: Close, Volumen, RSI, MACD, ATR, EMA20, EMA51</t>
   </si>
   <si>
-    <t>LSTM Clasica con ventanas de tiempo de 90 dias: Close, Volumen, RSI, MACD, ATR, EMA20, EMA52</t>
-  </si>
-  <si>
-    <t>LSTM Bidireccional con ventanas de tiempo de 90 dias: Close, Volumen, RSI, MACD, ATR, EMA20, EMA52</t>
+    <t>LSTM Clasica con ventanas de tiempo de 25 dias: Close, Volumen, RSI, MACD, ATR, EMA20, EMA52</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capa 1: 32 Neuronas para no retornar secuencias 
+Capa 2: Un dropout del 40% para apagar neuronas aleatoriamente y prevenir el sobreajuste
+ Capa 3: Una capa densa de 16 neuronas con activacion RELU
+Capa 4 (salida): una capa densa de 1 neurona </t>
+  </si>
+  <si>
+    <t>LSTM Bidireccional con ventanas de tiempo de 25 dias: Close, Volumen, RSI, MACD, ATR, EMA20, EMA52</t>
+  </si>
+  <si>
+    <t>CNN con ventanas de tiempo de 90 dias: Close, Volumen, RSI, MACD, ATR, EMA20, EMA50</t>
   </si>
 </sst>
 </file>
@@ -480,15 +490,21 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor theme="0" tint="-0.14999847407452621"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -496,11 +512,22 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -512,6 +539,25 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="22" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -556,9 +602,9 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{17DD9F00-2A82-4A5D-A129-DC1A3966A506}" name="Tabla1" displayName="Tabla1" ref="B1:E14" totalsRowShown="0">
   <autoFilter ref="B1:E14" xr:uid="{17DD9F00-2A82-4A5D-A129-DC1A3966A506}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{A219EF1F-5F03-44BB-94D9-DDF84B5D15C2}" name="Descripcion" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{F2DDE521-31A0-4967-A63D-8E3F5E6ED67C}" name=" Caracteristicas" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{2FB7966A-C401-40F8-9DC1-33ADC97693CD}" name="Fecha de ejecucion" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{A219EF1F-5F03-44BB-94D9-DDF84B5D15C2}" name="Descripcion" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{F2DDE521-31A0-4967-A63D-8E3F5E6ED67C}" name=" Caracteristicas" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{2FB7966A-C401-40F8-9DC1-33ADC97693CD}" name="Fecha de ejecucion" dataDxfId="0"/>
     <tableColumn id="4" xr3:uid="{A19B35B0-35FB-4491-9788-07CC4387A7B2}" name="Grafica"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -569,9 +615,9 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{76FB69AF-82F3-47A8-80EA-3563E28A1970}" name="Tabla13" displayName="Tabla13" ref="B1:E14" totalsRowShown="0">
   <autoFilter ref="B1:E14" xr:uid="{76FB69AF-82F3-47A8-80EA-3563E28A1970}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{0A114052-5782-45CC-9E5D-CC04A9FD2372}" name="Descripcion" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{9F71BC4A-3F7C-4E8A-AF6E-2CD68C6A137B}" name=" Caracteristicas" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{E6F6E4ED-91D0-4818-8F23-52323C2D1126}" name="Fecha de ejecucion" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{0A114052-5782-45CC-9E5D-CC04A9FD2372}" name="Descripcion" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{9F71BC4A-3F7C-4E8A-AF6E-2CD68C6A137B}" name=" Caracteristicas" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{E6F6E4ED-91D0-4818-8F23-52323C2D1126}" name="Fecha de ejecucion" dataDxfId="3"/>
     <tableColumn id="4" xr3:uid="{0B1A018E-7C86-49CD-A15E-3842F058E12A}" name="Grafica"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -950,7 +996,7 @@
         <v>18</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="D4" s="2">
         <v>46116.984027777777</v>
@@ -1024,7 +1070,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="17.6640625" customWidth="1"/>
-    <col min="3" max="3" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.44140625" customWidth="1"/>
     <col min="4" max="4" width="19.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1042,7 +1088,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="2:5" ht="244.8">
+    <row r="2" spans="2:5" ht="158.4">
       <c r="B2" s="1" t="s">
         <v>5</v>
       </c>
@@ -1056,7 +1102,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="2:5" ht="244.8">
+    <row r="3" spans="2:5" ht="158.4">
       <c r="B3" s="1" t="s">
         <v>15</v>
       </c>
@@ -1070,12 +1116,12 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="2:5" ht="244.8">
+    <row r="4" spans="2:5" ht="158.4">
       <c r="B4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>4</v>
       </c>
       <c r="D4" s="2">
         <v>46116</v>
@@ -1145,6 +1191,61 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E55F091-AE40-4613-85E2-B6C210B704C9}">
+  <dimension ref="B1:E4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="2" max="2" width="29.21875" customWidth="1"/>
+    <col min="3" max="3" width="25.5546875" customWidth="1"/>
+    <col min="4" max="4" width="17.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:5">
+      <c r="B1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="2:5" ht="171.6" customHeight="1">
+      <c r="B2" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="7">
+        <v>46116.545138888891</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5">
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="11"/>
+    </row>
+    <row r="4" spans="2:5">
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CC70B30-BC9C-4CE1-81DA-6046A0FA93C5}">
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>

</xml_diff>